<commit_message>
Publica matrices MIP auditables V3
</commit_message>
<xml_diff>
--- a/validacion_matematica_mip.xlsx
+++ b/validacion_matematica_mip.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="75">
   <si>
     <t>pais</t>
   </si>
@@ -58,6 +58,12 @@
     <t>CI_importado_total</t>
   </si>
   <si>
+    <t>ajuste_intermedio_neg_count</t>
+  </si>
+  <si>
+    <t>ajuste_intermedio_min</t>
+  </si>
+  <si>
     <t>oferta_vs_demanda_abs_max</t>
   </si>
   <si>
@@ -70,9 +76,27 @@
     <t>Lf_vs_g_rel_max</t>
   </si>
   <si>
+    <t>demanda_final_neg_count</t>
+  </si>
+  <si>
     <t>demanda_final_neg_share</t>
   </si>
   <si>
+    <t>demanda_final_min</t>
+  </si>
+  <si>
+    <t>VA_neg_count</t>
+  </si>
+  <si>
+    <t>VA_min</t>
+  </si>
+  <si>
+    <t>VA_residual_neg_count</t>
+  </si>
+  <si>
+    <t>VA_residual_min</t>
+  </si>
+  <si>
     <t>validacion_estructural</t>
   </si>
   <si>
@@ -100,6 +124,9 @@
     <t>uruguay_cou</t>
   </si>
   <si>
+    <t>uruguay_cou_2012</t>
+  </si>
+  <si>
     <t>data\processed\argentina\mip_argentina_2004.xlsx</t>
   </si>
   <si>
@@ -203,6 +230,9 @@
   </si>
   <si>
     <t>data\processed\uruguay_cou\mip_uruguay_cou_2017.xlsx</t>
+  </si>
+  <si>
+    <t>data\processed\uruguay_cou_2012\mip_uruguay_cou_2012_2012.xlsx</t>
   </si>
   <si>
     <t>OK</t>
@@ -215,16 +245,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -240,7 +262,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -248,30 +270,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,83 +570,107 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:AC37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:21">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" spans="1:29">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:29">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B2">
         <v>2004</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D2">
         <v>162</v>
@@ -678,36 +706,60 @@
         <v>9888382.594520949</v>
       </c>
       <c r="O2">
+        <v>23</v>
+      </c>
+      <c r="P2">
+        <v>-22678562.44191631</v>
+      </c>
+      <c r="Q2">
         <v>2.235174179077148E-08</v>
       </c>
-      <c r="P2">
+      <c r="R2">
         <v>8.703795318445035E-16</v>
       </c>
-      <c r="Q2">
+      <c r="S2">
         <v>1.490116119384766E-08</v>
       </c>
-      <c r="R2">
+      <c r="T2">
         <v>1.476489642827825E-15</v>
       </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2" t="s">
-        <v>63</v>
-      </c>
-      <c r="U2" t="s">
-        <v>63</v>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>2631.880934567059</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>2631.88093456706</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:29">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B3">
         <v>2018</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D3">
         <v>107</v>
@@ -743,36 +795,60 @@
         <v>1839713047.886877</v>
       </c>
       <c r="O3">
+        <v>8</v>
+      </c>
+      <c r="P3">
+        <v>-226126268.6606633</v>
+      </c>
+      <c r="Q3">
         <v>4.76837158203125E-07</v>
       </c>
-      <c r="P3">
+      <c r="R3">
         <v>1.017338214050006E-15</v>
       </c>
-      <c r="Q3">
+      <c r="S3">
         <v>5.960464477539062E-07</v>
       </c>
-      <c r="R3">
+      <c r="T3">
         <v>1.015682346479084E-15</v>
       </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3" t="s">
-        <v>63</v>
-      </c>
-      <c r="U3" t="s">
-        <v>63</v>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>1138797.60114376</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>1138797.60114376</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:29">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B4">
         <v>2019</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D4">
         <v>107</v>
@@ -808,36 +884,60 @@
         <v>2590768735.870364</v>
       </c>
       <c r="O4">
+        <v>10</v>
+      </c>
+      <c r="P4">
+        <v>-360237808.8982931</v>
+      </c>
+      <c r="Q4">
         <v>9.5367431640625E-07</v>
       </c>
-      <c r="P4">
+      <c r="R4">
         <v>8.165191710165035E-16</v>
       </c>
-      <c r="Q4">
+      <c r="S4">
         <v>7.152557373046875E-07</v>
       </c>
-      <c r="R4">
+      <c r="T4">
         <v>1.194638398520583E-15</v>
       </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4" t="s">
-        <v>63</v>
-      </c>
-      <c r="U4" t="s">
-        <v>63</v>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>1080546.527742543</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>1080546.527742543</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:29">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B5">
         <v>2020</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D5">
         <v>107</v>
@@ -873,36 +973,60 @@
         <v>3135231048.521698</v>
       </c>
       <c r="O5">
+        <v>8</v>
+      </c>
+      <c r="P5">
+        <v>-902599433.6951659</v>
+      </c>
+      <c r="Q5">
         <v>7.152557373046875E-07</v>
       </c>
-      <c r="P5">
+      <c r="R5">
         <v>1.028111652848961E-15</v>
       </c>
-      <c r="Q5">
+      <c r="S5">
         <v>1.430511474609375E-06</v>
       </c>
-      <c r="R5">
+      <c r="T5">
         <v>1.260959104652176E-15</v>
       </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5" t="s">
-        <v>63</v>
-      </c>
-      <c r="U5" t="s">
-        <v>63</v>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>1337871.655595163</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
+        <v>1337871.655595163</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:29">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B6">
         <v>2021</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D6">
         <v>107</v>
@@ -938,36 +1062,60 @@
         <v>5729027778.532877</v>
       </c>
       <c r="O6">
-        <v>1.9073486328125E-06</v>
+        <v>10</v>
       </c>
       <c r="P6">
-        <v>1.215517039538581E-15</v>
+        <v>-1590042819.174856</v>
       </c>
       <c r="Q6">
         <v>1.9073486328125E-06</v>
       </c>
       <c r="R6">
+        <v>1.215517039538581E-15</v>
+      </c>
+      <c r="S6">
+        <v>1.9073486328125E-06</v>
+      </c>
+      <c r="T6">
         <v>1.067366612072952E-15</v>
       </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-      <c r="T6" t="s">
-        <v>63</v>
-      </c>
-      <c r="U6" t="s">
-        <v>63</v>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>1246063.610381016</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>1246063.610381016</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:29">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B7">
         <v>2022</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D7">
         <v>107</v>
@@ -1003,36 +1151,60 @@
         <v>9916788550.378954</v>
       </c>
       <c r="O7">
-        <v>1.9073486328125E-06</v>
+        <v>9</v>
       </c>
       <c r="P7">
-        <v>7.669169106925529E-16</v>
+        <v>-2566666688.55542</v>
       </c>
       <c r="Q7">
         <v>1.9073486328125E-06</v>
       </c>
       <c r="R7">
+        <v>7.669169106925529E-16</v>
+      </c>
+      <c r="S7">
+        <v>1.9073486328125E-06</v>
+      </c>
+      <c r="T7">
         <v>8.505257508646007E-16</v>
       </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7" t="s">
-        <v>63</v>
-      </c>
-      <c r="U7" t="s">
-        <v>63</v>
+      <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>2259611.439475</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>2259611.439474999</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:29">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B8">
         <v>1997</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D8">
         <v>124</v>
@@ -1068,36 +1240,60 @@
         <v>0</v>
       </c>
       <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
         <v>3.725290298461914E-09</v>
       </c>
-      <c r="P8">
+      <c r="R8">
         <v>4.997123596493052E-16</v>
       </c>
-      <c r="Q8">
+      <c r="S8">
         <v>1710.538463994861</v>
       </c>
-      <c r="R8">
+      <c r="T8">
         <v>0.0008810551068959044</v>
       </c>
-      <c r="S8">
-        <v>0</v>
-      </c>
-      <c r="T8" t="s">
-        <v>63</v>
-      </c>
-      <c r="U8" t="s">
-        <v>64</v>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>3.585591912269592E-08</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>29736.41303924712</v>
+      </c>
+      <c r="Z8">
+        <v>0</v>
+      </c>
+      <c r="AA8">
+        <v>30013.40383325176</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:29">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B9">
         <v>2010</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="D9">
         <v>68</v>
@@ -1133,36 +1329,60 @@
         <v>265357.0640956726</v>
       </c>
       <c r="O9">
+        <v>19</v>
+      </c>
+      <c r="P9">
+        <v>-34468.07511866713</v>
+      </c>
+      <c r="Q9">
         <v>568.4045890633715</v>
       </c>
-      <c r="P9">
+      <c r="R9">
         <v>0.001053836421329765</v>
       </c>
-      <c r="Q9">
+      <c r="S9">
         <v>655.7265491787111</v>
       </c>
-      <c r="R9">
+      <c r="T9">
         <v>0.001215733534270193</v>
       </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
-      <c r="T9" t="s">
-        <v>63</v>
-      </c>
-      <c r="U9" t="s">
-        <v>64</v>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>215.6507861359235</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
+      <c r="Y9">
+        <v>3408</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
+        <v>3408</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:29">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <v>2011</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D10">
         <v>68</v>
@@ -1198,36 +1418,60 @@
         <v>301998.6004792693</v>
       </c>
       <c r="O10">
+        <v>18</v>
+      </c>
+      <c r="P10">
+        <v>-45280.53271581482</v>
+      </c>
+      <c r="Q10">
         <v>787.7762729106471</v>
       </c>
-      <c r="P10">
+      <c r="R10">
         <v>0.001264685308805138</v>
       </c>
-      <c r="Q10">
+      <c r="S10">
         <v>915.2956661685603</v>
       </c>
-      <c r="R10">
+      <c r="T10">
         <v>0.001469403207511539</v>
       </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-      <c r="T10" t="s">
-        <v>63</v>
-      </c>
-      <c r="U10" t="s">
-        <v>64</v>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>249.679197757909</v>
+      </c>
+      <c r="X10">
+        <v>1</v>
+      </c>
+      <c r="Y10">
+        <v>-10202</v>
+      </c>
+      <c r="Z10">
+        <v>1</v>
+      </c>
+      <c r="AA10">
+        <v>-10202.00000000003</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:21">
+    <row r="11" spans="1:29">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B11">
         <v>2012</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="D11">
         <v>68</v>
@@ -1263,36 +1507,60 @@
         <v>342833.5955653188</v>
       </c>
       <c r="O11">
+        <v>18</v>
+      </c>
+      <c r="P11">
+        <v>-54019.0975862894</v>
+      </c>
+      <c r="Q11">
         <v>799.3443168383092</v>
       </c>
-      <c r="P11">
+      <c r="R11">
         <v>0.001104228404764108</v>
       </c>
-      <c r="Q11">
+      <c r="S11">
         <v>926.085863463697</v>
       </c>
-      <c r="R11">
+      <c r="T11">
         <v>0.001279311423307414</v>
       </c>
-      <c r="S11">
-        <v>0</v>
-      </c>
-      <c r="T11" t="s">
-        <v>63</v>
-      </c>
-      <c r="U11" t="s">
-        <v>64</v>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>223.82068590636</v>
+      </c>
+      <c r="X11">
+        <v>1</v>
+      </c>
+      <c r="Y11">
+        <v>-27152</v>
+      </c>
+      <c r="Z11">
+        <v>1</v>
+      </c>
+      <c r="AA11">
+        <v>-27152</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:29">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B12">
         <v>2013</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D12">
         <v>68</v>
@@ -1328,36 +1596,60 @@
         <v>378788.9518083158</v>
       </c>
       <c r="O12">
+        <v>18</v>
+      </c>
+      <c r="P12">
+        <v>-65073.62717264631</v>
+      </c>
+      <c r="Q12">
         <v>998.4611635631882</v>
       </c>
-      <c r="P12">
+      <c r="R12">
         <v>0.001214000964871255</v>
       </c>
-      <c r="Q12">
+      <c r="S12">
         <v>1163.741865767981</v>
       </c>
-      <c r="R12">
+      <c r="T12">
         <v>0.00141496114166487</v>
       </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
-      <c r="T12" t="s">
-        <v>63</v>
-      </c>
-      <c r="U12" t="s">
-        <v>64</v>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>390.4927428090983</v>
+      </c>
+      <c r="X12">
+        <v>1</v>
+      </c>
+      <c r="Y12">
+        <v>-28223</v>
+      </c>
+      <c r="Z12">
+        <v>1</v>
+      </c>
+      <c r="AA12">
+        <v>-28222.99999999999</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:29">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B13">
         <v>2014</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D13">
         <v>68</v>
@@ -1393,36 +1685,60 @@
         <v>418367.5884969411</v>
       </c>
       <c r="O13">
+        <v>20</v>
+      </c>
+      <c r="P13">
+        <v>-69598.87814064437</v>
+      </c>
+      <c r="Q13">
         <v>694.8371658106335</v>
       </c>
-      <c r="P13">
+      <c r="R13">
         <v>0.0007607825587890249</v>
       </c>
-      <c r="Q13">
+      <c r="S13">
         <v>806.0285520588513</v>
       </c>
-      <c r="R13">
+      <c r="T13">
         <v>0.0008825268630772505</v>
       </c>
-      <c r="S13">
-        <v>0</v>
-      </c>
-      <c r="T13" t="s">
-        <v>63</v>
-      </c>
-      <c r="U13" t="s">
-        <v>64</v>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>425.980176712754</v>
+      </c>
+      <c r="X13">
+        <v>1</v>
+      </c>
+      <c r="Y13">
+        <v>-16729</v>
+      </c>
+      <c r="Z13">
+        <v>1</v>
+      </c>
+      <c r="AA13">
+        <v>-16729</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:21">
+    <row r="14" spans="1:29">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>2015</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D14">
         <v>68</v>
@@ -1458,36 +1774,60 @@
         <v>446677.1926265535</v>
       </c>
       <c r="O14">
+        <v>19</v>
+      </c>
+      <c r="P14">
+        <v>-78531.9954223911</v>
+      </c>
+      <c r="Q14">
         <v>224.4737316915998</v>
       </c>
-      <c r="P14">
+      <c r="R14">
         <v>0.000508180337461277</v>
       </c>
-      <c r="Q14">
+      <c r="S14">
         <v>266.5394776551984</v>
       </c>
-      <c r="R14">
+      <c r="T14">
         <v>0.0005429579563502418</v>
       </c>
-      <c r="S14">
-        <v>0</v>
-      </c>
-      <c r="T14" t="s">
-        <v>63</v>
-      </c>
-      <c r="U14" t="s">
-        <v>64</v>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>440.072707192931</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>4258</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>4258</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:21">
+    <row r="15" spans="1:29">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>2016</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D15">
         <v>68</v>
@@ -1523,36 +1863,60 @@
         <v>377797.5402644395</v>
       </c>
       <c r="O15">
+        <v>23</v>
+      </c>
+      <c r="P15">
+        <v>-86675.11045879175</v>
+      </c>
+      <c r="Q15">
         <v>21.58701042598113</v>
       </c>
-      <c r="P15">
+      <c r="R15">
         <v>2.196936525894786E-05</v>
       </c>
-      <c r="Q15">
+      <c r="S15">
         <v>25.05347653967328</v>
       </c>
-      <c r="R15">
+      <c r="T15">
         <v>2.549723033644884E-05</v>
       </c>
-      <c r="S15">
-        <v>0</v>
-      </c>
-      <c r="T15" t="s">
-        <v>63</v>
-      </c>
-      <c r="U15" t="s">
-        <v>64</v>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>480.9925597825006</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>3855</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>3855.000000000001</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:21">
+    <row r="16" spans="1:29">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B16">
         <v>2017</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="D16">
         <v>68</v>
@@ -1588,36 +1952,60 @@
         <v>364522.4860841213</v>
       </c>
       <c r="O16">
+        <v>22</v>
+      </c>
+      <c r="P16">
+        <v>-97054.41987754889</v>
+      </c>
+      <c r="Q16">
         <v>602.4990921429126</v>
       </c>
-      <c r="P16">
+      <c r="R16">
         <v>0.0005745479108289929</v>
       </c>
-      <c r="Q16">
+      <c r="S16">
         <v>706.8542623416288</v>
       </c>
-      <c r="R16">
+      <c r="T16">
         <v>0.0006740618284493942</v>
       </c>
-      <c r="S16">
-        <v>0</v>
-      </c>
-      <c r="T16" t="s">
-        <v>63</v>
-      </c>
-      <c r="U16" t="s">
-        <v>64</v>
+      <c r="U16">
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <v>0</v>
+      </c>
+      <c r="W16">
+        <v>474.6436384931367</v>
+      </c>
+      <c r="X16">
+        <v>0</v>
+      </c>
+      <c r="Y16">
+        <v>3161</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+      <c r="AA16">
+        <v>3161.000000000003</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:21">
+    <row r="17" spans="1:29">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B17">
         <v>2018</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="D17">
         <v>68</v>
@@ -1653,36 +2041,60 @@
         <v>495901.5003305521</v>
       </c>
       <c r="O17">
-        <v>4.656612873077393E-10</v>
+        <v>19</v>
       </c>
       <c r="P17">
-        <v>5.838090625277251E-16</v>
+        <v>-104750.439988568</v>
       </c>
       <c r="Q17">
         <v>4.656612873077393E-10</v>
       </c>
       <c r="R17">
+        <v>5.838090625277251E-16</v>
+      </c>
+      <c r="S17">
+        <v>4.656612873077393E-10</v>
+      </c>
+      <c r="T17">
         <v>5.765551328127705E-16</v>
       </c>
-      <c r="S17">
-        <v>0</v>
-      </c>
-      <c r="T17" t="s">
-        <v>63</v>
-      </c>
-      <c r="U17" t="s">
-        <v>63</v>
+      <c r="U17">
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>496.5330684426606</v>
+      </c>
+      <c r="X17">
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <v>3582</v>
+      </c>
+      <c r="Z17">
+        <v>0</v>
+      </c>
+      <c r="AA17">
+        <v>3582</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:21">
+    <row r="18" spans="1:29">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B18">
         <v>2019</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D18">
         <v>68</v>
@@ -1718,36 +2130,60 @@
         <v>538025.4537202606</v>
       </c>
       <c r="O18">
+        <v>20</v>
+      </c>
+      <c r="P18">
+        <v>-121733.4284180765</v>
+      </c>
+      <c r="Q18">
         <v>2.328306436538696E-10</v>
       </c>
-      <c r="P18">
+      <c r="R18">
         <v>5.356270328462475E-16</v>
       </c>
-      <c r="Q18">
+      <c r="S18">
         <v>3.492459654808044E-10</v>
       </c>
-      <c r="R18">
+      <c r="T18">
         <v>8.333833619223625E-16</v>
       </c>
-      <c r="S18">
-        <v>0</v>
-      </c>
-      <c r="T18" t="s">
-        <v>63</v>
-      </c>
-      <c r="U18" t="s">
-        <v>63</v>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+      <c r="W18">
+        <v>546.3796691584467</v>
+      </c>
+      <c r="X18">
+        <v>0</v>
+      </c>
+      <c r="Y18">
+        <v>3789</v>
+      </c>
+      <c r="Z18">
+        <v>0</v>
+      </c>
+      <c r="AA18">
+        <v>3789.000000000002</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:29">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B19">
         <v>2020</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D19">
         <v>68</v>
@@ -1783,36 +2219,60 @@
         <v>567057.7066328113</v>
       </c>
       <c r="O19">
+        <v>19</v>
+      </c>
+      <c r="P19">
+        <v>-134974.1019460761</v>
+      </c>
+      <c r="Q19">
         <v>184.9745980203152</v>
       </c>
-      <c r="P19">
+      <c r="R19">
         <v>0.0001505080939887886</v>
       </c>
-      <c r="Q19">
+      <c r="S19">
         <v>217.3657415492926</v>
       </c>
-      <c r="R19">
+      <c r="T19">
         <v>0.0001768637629662568</v>
       </c>
-      <c r="S19">
-        <v>0</v>
-      </c>
-      <c r="T19" t="s">
-        <v>63</v>
-      </c>
-      <c r="U19" t="s">
-        <v>64</v>
+      <c r="U19">
+        <v>0</v>
+      </c>
+      <c r="V19">
+        <v>0</v>
+      </c>
+      <c r="W19">
+        <v>547.268735049141</v>
+      </c>
+      <c r="X19">
+        <v>0</v>
+      </c>
+      <c r="Y19">
+        <v>3834</v>
+      </c>
+      <c r="Z19">
+        <v>0</v>
+      </c>
+      <c r="AA19">
+        <v>3833.999999999998</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:29">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B20">
         <v>2021</v>
       </c>
       <c r="C20" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="D20">
         <v>68</v>
@@ -1848,36 +2308,60 @@
         <v>926717.306588684</v>
       </c>
       <c r="O20">
+        <v>16</v>
+      </c>
+      <c r="P20">
+        <v>-137760.1279216045</v>
+      </c>
+      <c r="Q20">
         <v>285.3846563701518</v>
       </c>
-      <c r="P20">
+      <c r="R20">
         <v>0.0001978560899968814</v>
       </c>
-      <c r="Q20">
+      <c r="S20">
         <v>334.3216072747018</v>
       </c>
-      <c r="R20">
+      <c r="T20">
         <v>0.0002317838907605818</v>
       </c>
-      <c r="S20">
-        <v>0</v>
-      </c>
-      <c r="T20" t="s">
-        <v>63</v>
-      </c>
-      <c r="U20" t="s">
-        <v>64</v>
+      <c r="U20">
+        <v>0</v>
+      </c>
+      <c r="V20">
+        <v>0</v>
+      </c>
+      <c r="W20">
+        <v>560.5603185020369</v>
+      </c>
+      <c r="X20">
+        <v>0</v>
+      </c>
+      <c r="Y20">
+        <v>3073</v>
+      </c>
+      <c r="Z20">
+        <v>0</v>
+      </c>
+      <c r="AA20">
+        <v>3073.000000000007</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:21">
+    <row r="21" spans="1:29">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B21">
         <v>2000</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="D21">
         <v>51</v>
@@ -1913,36 +2397,60 @@
         <v>163728.8372825221</v>
       </c>
       <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
         <v>423.5260419981205</v>
       </c>
-      <c r="P21">
+      <c r="R21">
         <v>0.002721157326835654</v>
       </c>
-      <c r="Q21">
+      <c r="S21">
         <v>456.7713921025279</v>
       </c>
-      <c r="R21">
+      <c r="T21">
         <v>0.002934758898047244</v>
       </c>
-      <c r="S21">
-        <v>0</v>
-      </c>
-      <c r="T21" t="s">
-        <v>63</v>
-      </c>
-      <c r="U21" t="s">
-        <v>64</v>
+      <c r="U21">
+        <v>0</v>
+      </c>
+      <c r="V21">
+        <v>0</v>
+      </c>
+      <c r="W21">
+        <v>452.6602163484574</v>
+      </c>
+      <c r="X21">
+        <v>0</v>
+      </c>
+      <c r="Y21">
+        <v>463.714128762466</v>
+      </c>
+      <c r="Z21">
+        <v>0</v>
+      </c>
+      <c r="AA21">
+        <v>463.7141287624581</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:21">
+    <row r="22" spans="1:29">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B22">
         <v>2001</v>
       </c>
       <c r="C22" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="D22">
         <v>51</v>
@@ -1978,36 +2486,60 @@
         <v>199760.1694606353</v>
       </c>
       <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
         <v>468.8965698834218</v>
       </c>
-      <c r="P22">
+      <c r="R22">
         <v>0.004335383955587383</v>
       </c>
-      <c r="Q22">
+      <c r="S22">
         <v>519.6551209768222</v>
       </c>
-      <c r="R22">
+      <c r="T22">
         <v>0.004804693867736883</v>
       </c>
-      <c r="S22">
-        <v>0</v>
-      </c>
-      <c r="T22" t="s">
-        <v>63</v>
-      </c>
-      <c r="U22" t="s">
-        <v>64</v>
+      <c r="U22">
+        <v>0</v>
+      </c>
+      <c r="V22">
+        <v>0</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>0</v>
+      </c>
+      <c r="Y22">
+        <v>511.087891554102</v>
+      </c>
+      <c r="Z22">
+        <v>0</v>
+      </c>
+      <c r="AA22">
+        <v>511.0878915541057</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:21">
+    <row r="23" spans="1:29">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B23">
         <v>2002</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D23">
         <v>51</v>
@@ -2043,36 +2575,60 @@
         <v>223970.7016156241</v>
       </c>
       <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
         <v>463.0990200235974</v>
       </c>
-      <c r="P23">
+      <c r="R23">
         <v>0.00312648498607125</v>
       </c>
-      <c r="Q23">
+      <c r="S23">
         <v>529.854376289004</v>
       </c>
-      <c r="R23">
+      <c r="T23">
         <v>0.003577165315934604</v>
       </c>
-      <c r="S23">
-        <v>0</v>
-      </c>
-      <c r="T23" t="s">
-        <v>63</v>
-      </c>
-      <c r="U23" t="s">
-        <v>64</v>
+      <c r="U23">
+        <v>0</v>
+      </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="Y23">
+        <v>503.802692998641</v>
+      </c>
+      <c r="Z23">
+        <v>0</v>
+      </c>
+      <c r="AA23">
+        <v>503.8026929986431</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="24" spans="1:21">
+    <row r="24" spans="1:29">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B24">
         <v>2003</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="D24">
         <v>51</v>
@@ -2108,36 +2664,60 @@
         <v>250589.541394027</v>
       </c>
       <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
         <v>572.2698159218126</v>
       </c>
-      <c r="P24">
+      <c r="R24">
         <v>0.002354598184841582</v>
       </c>
-      <c r="Q24">
+      <c r="S24">
         <v>621.1031355652958</v>
       </c>
-      <c r="R24">
+      <c r="T24">
         <v>0.002555522368842306</v>
       </c>
-      <c r="S24">
-        <v>0</v>
-      </c>
-      <c r="T24" t="s">
-        <v>63</v>
-      </c>
-      <c r="U24" t="s">
-        <v>64</v>
+      <c r="U24">
+        <v>0</v>
+      </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+      <c r="W24">
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
+      <c r="Y24">
+        <v>955.423608665425</v>
+      </c>
+      <c r="Z24">
+        <v>0</v>
+      </c>
+      <c r="AA24">
+        <v>955.4236086654303</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:21">
+    <row r="25" spans="1:29">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B25">
         <v>2004</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D25">
         <v>51</v>
@@ -2173,36 +2753,60 @@
         <v>292993.2656904903</v>
       </c>
       <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
         <v>603.9112367413472</v>
       </c>
-      <c r="P25">
+      <c r="R25">
         <v>0.002132696365869464</v>
       </c>
-      <c r="Q25">
+      <c r="S25">
         <v>657.1939591109985</v>
       </c>
-      <c r="R25">
+      <c r="T25">
         <v>0.00232086287354128</v>
       </c>
-      <c r="S25">
-        <v>0</v>
-      </c>
-      <c r="T25" t="s">
-        <v>63</v>
-      </c>
-      <c r="U25" t="s">
-        <v>64</v>
+      <c r="U25">
+        <v>0</v>
+      </c>
+      <c r="V25">
+        <v>0</v>
+      </c>
+      <c r="W25">
+        <v>0</v>
+      </c>
+      <c r="X25">
+        <v>0</v>
+      </c>
+      <c r="Y25">
+        <v>1009.95926338168</v>
+      </c>
+      <c r="Z25">
+        <v>0</v>
+      </c>
+      <c r="AA25">
+        <v>1009.959263381683</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:21">
+    <row r="26" spans="1:29">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B26">
         <v>2005</v>
       </c>
       <c r="C26" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D26">
         <v>51</v>
@@ -2238,36 +2842,60 @@
         <v>300063.9490641863</v>
       </c>
       <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26">
         <v>774.0081208376796</v>
       </c>
-      <c r="P26">
+      <c r="R26">
         <v>0.002345889803039813</v>
       </c>
-      <c r="Q26">
+      <c r="S26">
         <v>844.8867201150861</v>
       </c>
-      <c r="R26">
+      <c r="T26">
         <v>0.002560711041761006</v>
       </c>
-      <c r="S26">
-        <v>0</v>
-      </c>
-      <c r="T26" t="s">
-        <v>63</v>
-      </c>
-      <c r="U26" t="s">
-        <v>64</v>
+      <c r="U26">
+        <v>0</v>
+      </c>
+      <c r="V26">
+        <v>0</v>
+      </c>
+      <c r="W26">
+        <v>0</v>
+      </c>
+      <c r="X26">
+        <v>0</v>
+      </c>
+      <c r="Y26">
+        <v>1074.30338163792</v>
+      </c>
+      <c r="Z26">
+        <v>0</v>
+      </c>
+      <c r="AA26">
+        <v>1074.303381637912</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:21">
+    <row r="27" spans="1:29">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <v>2006</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D27">
         <v>51</v>
@@ -2303,36 +2931,60 @@
         <v>315938.3044747321</v>
       </c>
       <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27">
+        <v>-70.54599560104361</v>
+      </c>
+      <c r="Q27">
         <v>849.009810589836</v>
       </c>
-      <c r="P27">
+      <c r="R27">
         <v>0.002266818499511618</v>
       </c>
-      <c r="Q27">
+      <c r="S27">
         <v>928.4832096964237</v>
       </c>
-      <c r="R27">
+      <c r="T27">
         <v>0.002479008946626388</v>
       </c>
-      <c r="S27">
-        <v>0</v>
-      </c>
-      <c r="T27" t="s">
-        <v>63</v>
-      </c>
-      <c r="U27" t="s">
-        <v>64</v>
+      <c r="U27">
+        <v>0</v>
+      </c>
+      <c r="V27">
+        <v>0</v>
+      </c>
+      <c r="W27">
+        <v>0</v>
+      </c>
+      <c r="X27">
+        <v>0</v>
+      </c>
+      <c r="Y27">
+        <v>1267.92926028247</v>
+      </c>
+      <c r="Z27">
+        <v>0</v>
+      </c>
+      <c r="AA27">
+        <v>1267.929260282477</v>
+      </c>
+      <c r="AB27" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC27" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:21">
+    <row r="28" spans="1:29">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B28">
         <v>2007</v>
       </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D28">
         <v>51</v>
@@ -2368,36 +3020,60 @@
         <v>347764.7604630886</v>
       </c>
       <c r="O28">
+        <v>4</v>
+      </c>
+      <c r="P28">
+        <v>-1540.333394080684</v>
+      </c>
+      <c r="Q28">
         <v>1129.460600296792</v>
       </c>
-      <c r="P28">
+      <c r="R28">
         <v>0.002589907307863009</v>
       </c>
-      <c r="Q28">
+      <c r="S28">
         <v>1241.773817741836</v>
       </c>
-      <c r="R28">
+      <c r="T28">
         <v>0.002847446900261443</v>
       </c>
-      <c r="S28">
-        <v>0</v>
-      </c>
-      <c r="T28" t="s">
-        <v>63</v>
-      </c>
-      <c r="U28" t="s">
-        <v>64</v>
+      <c r="U28">
+        <v>0</v>
+      </c>
+      <c r="V28">
+        <v>0</v>
+      </c>
+      <c r="W28">
+        <v>490.1342912259377</v>
+      </c>
+      <c r="X28">
+        <v>0</v>
+      </c>
+      <c r="Y28">
+        <v>1310.69163025554</v>
+      </c>
+      <c r="Z28">
+        <v>0</v>
+      </c>
+      <c r="AA28">
+        <v>1310.69163025554</v>
+      </c>
+      <c r="AB28" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC28" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:21">
+    <row r="29" spans="1:29">
       <c r="A29" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B29">
         <v>2008</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D29">
         <v>51</v>
@@ -2433,36 +3109,60 @@
         <v>432399.9132605757</v>
       </c>
       <c r="O29">
+        <v>4</v>
+      </c>
+      <c r="P29">
+        <v>-2103.884834608309</v>
+      </c>
+      <c r="Q29">
         <v>1208.869434595399</v>
       </c>
-      <c r="P29">
+      <c r="R29">
         <v>0.002365243819252891</v>
       </c>
-      <c r="Q29">
+      <c r="S29">
         <v>1332.656584697485</v>
       </c>
-      <c r="R29">
+      <c r="T29">
         <v>0.002607442673242347</v>
       </c>
-      <c r="S29">
-        <v>0</v>
-      </c>
-      <c r="T29" t="s">
-        <v>63</v>
-      </c>
-      <c r="U29" t="s">
-        <v>64</v>
+      <c r="U29">
+        <v>0</v>
+      </c>
+      <c r="V29">
+        <v>0</v>
+      </c>
+      <c r="W29">
+        <v>739.3987407752509</v>
+      </c>
+      <c r="X29">
+        <v>0</v>
+      </c>
+      <c r="Y29">
+        <v>1644.14244847053</v>
+      </c>
+      <c r="Z29">
+        <v>0</v>
+      </c>
+      <c r="AA29">
+        <v>1644.142448470529</v>
+      </c>
+      <c r="AB29" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC29" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="30" spans="1:21">
+    <row r="30" spans="1:29">
       <c r="A30" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B30">
         <v>2009</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="D30">
         <v>51</v>
@@ -2498,36 +3198,60 @@
         <v>385803.7195056804</v>
       </c>
       <c r="O30">
+        <v>6</v>
+      </c>
+      <c r="P30">
+        <v>-4629.727207051419</v>
+      </c>
+      <c r="Q30">
         <v>1214.7142444239</v>
       </c>
-      <c r="P30">
+      <c r="R30">
         <v>0.002145869631775909</v>
       </c>
-      <c r="Q30">
+      <c r="S30">
         <v>1349.402535793371</v>
       </c>
-      <c r="R30">
+      <c r="T30">
         <v>0.002383805027308057</v>
       </c>
-      <c r="S30">
-        <v>0</v>
-      </c>
-      <c r="T30" t="s">
-        <v>63</v>
-      </c>
-      <c r="U30" t="s">
-        <v>64</v>
+      <c r="U30">
+        <v>0</v>
+      </c>
+      <c r="V30">
+        <v>0</v>
+      </c>
+      <c r="W30">
+        <v>177.3059107023601</v>
+      </c>
+      <c r="X30">
+        <v>0</v>
+      </c>
+      <c r="Y30">
+        <v>1626.28977832027</v>
+      </c>
+      <c r="Z30">
+        <v>0</v>
+      </c>
+      <c r="AA30">
+        <v>1626.289778320272</v>
+      </c>
+      <c r="AB30" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC30" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:21">
+    <row r="31" spans="1:29">
       <c r="A31" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B31">
         <v>2003</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D31">
         <v>20</v>
@@ -2569,30 +3293,54 @@
         <v>0</v>
       </c>
       <c r="Q31">
+        <v>0</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+      <c r="S31">
         <v>9.5367431640625E-07</v>
       </c>
-      <c r="R31">
+      <c r="T31">
         <v>4.378808426553387E-16</v>
       </c>
-      <c r="S31">
-        <v>0</v>
-      </c>
-      <c r="T31" t="s">
-        <v>63</v>
-      </c>
-      <c r="U31" t="s">
-        <v>64</v>
+      <c r="U31">
+        <v>0</v>
+      </c>
+      <c r="V31">
+        <v>0</v>
+      </c>
+      <c r="W31">
+        <v>0</v>
+      </c>
+      <c r="X31">
+        <v>0</v>
+      </c>
+      <c r="Y31">
+        <v>8990120</v>
+      </c>
+      <c r="Z31">
+        <v>0</v>
+      </c>
+      <c r="AA31">
+        <v>9153584</v>
+      </c>
+      <c r="AB31" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC31" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:21">
+    <row r="32" spans="1:29">
       <c r="A32" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B32">
         <v>2008</v>
       </c>
       <c r="C32" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D32">
         <v>262</v>
@@ -2628,36 +3376,60 @@
         <v>0</v>
       </c>
       <c r="O32">
+        <v>0</v>
+      </c>
+      <c r="P32">
+        <v>0</v>
+      </c>
+      <c r="Q32">
         <v>4.656612873077393E-10</v>
       </c>
-      <c r="P32">
+      <c r="R32">
         <v>4.153587537168728E-16</v>
       </c>
-      <c r="Q32">
+      <c r="S32">
         <v>3.492459654808044E-10</v>
       </c>
-      <c r="R32">
+      <c r="T32">
         <v>1.326250839504173E-15</v>
       </c>
-      <c r="S32">
+      <c r="U32">
+        <v>3</v>
+      </c>
+      <c r="V32">
         <v>0.01145038167938931</v>
       </c>
-      <c r="T32" t="s">
-        <v>63</v>
-      </c>
-      <c r="U32" t="s">
-        <v>64</v>
+      <c r="W32">
+        <v>-1629.63500000002</v>
+      </c>
+      <c r="X32">
+        <v>0</v>
+      </c>
+      <c r="Y32">
+        <v>9.381000000000002</v>
+      </c>
+      <c r="Z32">
+        <v>0</v>
+      </c>
+      <c r="AA32">
+        <v>9.267000000000001</v>
+      </c>
+      <c r="AB32" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC32" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:21">
+    <row r="33" spans="1:29">
       <c r="A33" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B33">
         <v>2013</v>
       </c>
       <c r="C33" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="D33">
         <v>262</v>
@@ -2693,36 +3465,60 @@
         <v>3898884.412</v>
       </c>
       <c r="O33">
+        <v>0</v>
+      </c>
+      <c r="P33">
+        <v>0</v>
+      </c>
+      <c r="Q33">
         <v>2.328306436538696E-10</v>
       </c>
-      <c r="P33">
+      <c r="R33">
         <v>4.297751578932477E-16</v>
       </c>
-      <c r="Q33">
+      <c r="S33">
         <v>2.693850547075272E-07</v>
       </c>
-      <c r="R33">
+      <c r="T33">
         <v>4.284818590404693E-12</v>
       </c>
-      <c r="S33">
+      <c r="U33">
+        <v>1</v>
+      </c>
+      <c r="V33">
         <v>0.003816793893129771</v>
       </c>
-      <c r="T33" t="s">
-        <v>63</v>
-      </c>
-      <c r="U33" t="s">
-        <v>64</v>
+      <c r="W33">
+        <v>-0.002999999550638677</v>
+      </c>
+      <c r="X33">
+        <v>0</v>
+      </c>
+      <c r="Y33">
+        <v>0</v>
+      </c>
+      <c r="Z33">
+        <v>0</v>
+      </c>
+      <c r="AA33">
+        <v>0</v>
+      </c>
+      <c r="AB33" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC33" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="34" spans="1:21">
+    <row r="34" spans="1:29">
       <c r="A34" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B34">
         <v>2018</v>
       </c>
       <c r="C34" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D34">
         <v>263</v>
@@ -2758,36 +3554,60 @@
         <v>7162500.963</v>
       </c>
       <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34">
+        <v>0</v>
+      </c>
+      <c r="Q34">
         <v>4.656612873077393E-10</v>
       </c>
-      <c r="P34">
+      <c r="R34">
         <v>7.67264506481741E-16</v>
       </c>
-      <c r="Q34">
+      <c r="S34">
         <v>3.012828528881073E-07</v>
       </c>
-      <c r="R34">
+      <c r="T34">
         <v>4.556388941836081E-12</v>
       </c>
-      <c r="S34">
-        <v>0</v>
-      </c>
-      <c r="T34" t="s">
-        <v>63</v>
-      </c>
-      <c r="U34" t="s">
-        <v>64</v>
+      <c r="U34">
+        <v>0</v>
+      </c>
+      <c r="V34">
+        <v>0</v>
+      </c>
+      <c r="W34">
+        <v>0</v>
+      </c>
+      <c r="X34">
+        <v>0</v>
+      </c>
+      <c r="Y34">
+        <v>0</v>
+      </c>
+      <c r="Z34">
+        <v>0</v>
+      </c>
+      <c r="AA34">
+        <v>0</v>
+      </c>
+      <c r="AB34" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:21">
+    <row r="35" spans="1:29">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B35">
         <v>2016</v>
       </c>
       <c r="C35" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="D35">
         <v>128</v>
@@ -2823,10 +3643,10 @@
         <v>0</v>
       </c>
       <c r="O35">
-        <v>8.256756700575352E-08</v>
+        <v>0</v>
       </c>
       <c r="P35">
-        <v>1.038996511523405E-12</v>
+        <v>0</v>
       </c>
       <c r="Q35">
         <v>8.256756700575352E-08</v>
@@ -2835,24 +3655,48 @@
         <v>1.038996511523405E-12</v>
       </c>
       <c r="S35">
-        <v>0</v>
-      </c>
-      <c r="T35" t="s">
-        <v>63</v>
-      </c>
-      <c r="U35" t="s">
-        <v>64</v>
+        <v>8.256756700575352E-08</v>
+      </c>
+      <c r="T35">
+        <v>1.038996511523405E-12</v>
+      </c>
+      <c r="U35">
+        <v>0</v>
+      </c>
+      <c r="V35">
+        <v>0</v>
+      </c>
+      <c r="W35">
+        <v>0</v>
+      </c>
+      <c r="X35">
+        <v>0</v>
+      </c>
+      <c r="Y35">
+        <v>7.66</v>
+      </c>
+      <c r="Z35">
+        <v>0</v>
+      </c>
+      <c r="AA35">
+        <v>12.61</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC35" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:21">
+    <row r="36" spans="1:29">
       <c r="A36" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B36">
         <v>2017</v>
       </c>
       <c r="C36" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D36">
         <v>95</v>
@@ -2888,25 +3732,138 @@
         <v>248046.07</v>
       </c>
       <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36">
+        <v>0</v>
+      </c>
+      <c r="Q36">
         <v>2.91038304567337E-11</v>
       </c>
-      <c r="P36">
+      <c r="R36">
         <v>6.450871763071315E-16</v>
       </c>
-      <c r="Q36">
+      <c r="S36">
         <v>5.820766091346741E-11</v>
       </c>
-      <c r="R36">
+      <c r="T36">
         <v>7.700799152212248E-16</v>
       </c>
-      <c r="S36">
+      <c r="U36">
+        <v>2</v>
+      </c>
+      <c r="V36">
         <v>0.02105263157894737</v>
       </c>
-      <c r="T36" t="s">
-        <v>63</v>
-      </c>
-      <c r="U36" t="s">
-        <v>64</v>
+      <c r="W36">
+        <v>-25062.16195323598</v>
+      </c>
+      <c r="X36">
+        <v>1</v>
+      </c>
+      <c r="Y36">
+        <v>-780.1151887383123</v>
+      </c>
+      <c r="Z36">
+        <v>1</v>
+      </c>
+      <c r="AA36">
+        <v>-780.1151887383114</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC36" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:29">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>2012</v>
+      </c>
+      <c r="C37" t="s">
+        <v>72</v>
+      </c>
+      <c r="D37">
+        <v>107</v>
+      </c>
+      <c r="E37" t="b">
+        <v>1</v>
+      </c>
+      <c r="F37" t="b">
+        <v>1</v>
+      </c>
+      <c r="G37" t="b">
+        <v>1</v>
+      </c>
+      <c r="H37" t="b">
+        <v>1</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>1.387778780781446E-16</v>
+      </c>
+      <c r="K37">
+        <v>1.332267629550188E-15</v>
+      </c>
+      <c r="L37">
+        <v>119320.7977373219</v>
+      </c>
+      <c r="M37">
+        <v>1</v>
+      </c>
+      <c r="N37">
+        <v>0</v>
+      </c>
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37">
+        <v>0</v>
+      </c>
+      <c r="Q37">
+        <v>2.91038304567337E-11</v>
+      </c>
+      <c r="R37">
+        <v>1.008143985052256E-15</v>
+      </c>
+      <c r="S37">
+        <v>1.164153218269348E-10</v>
+      </c>
+      <c r="T37">
+        <v>1.25881434502794E-15</v>
+      </c>
+      <c r="U37">
+        <v>13</v>
+      </c>
+      <c r="V37">
+        <v>0.1214953271028037</v>
+      </c>
+      <c r="W37">
+        <v>-5983.84951657153</v>
+      </c>
+      <c r="X37">
+        <v>0</v>
+      </c>
+      <c r="Y37">
+        <v>0</v>
+      </c>
+      <c r="Z37">
+        <v>1</v>
+      </c>
+      <c r="AA37">
+        <v>-177.9506604436215</v>
+      </c>
+      <c r="AB37" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC37" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>